<commit_message>
WA list rebuilt: clean 3-sheet separation (replied / never-contacted / already-contacted)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WA Pending (send after unban)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1-REPLIED (send first)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2-NEVER contacted (cold)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3-CONTACTED on old number" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +42,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00808080"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,9 +67,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,16 +437,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,107 +461,242 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Phone</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>History</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>IG Handle</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Action</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>L001</t>
+          <t>L007</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Golden Kyu Barcelona</t>
+          <t>Team Duramuk</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>351967734557</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>+34670425918</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>info@goldenkyu.com</t>
+          <t>Conversation existed on old number</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>@goldenkyu_bcn</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM + WA + email sent</t>
+          <t>REPLIED before - re-contact first</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>L002</t>
+          <t>L078</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kick Barcelona</t>
+          <t>Scorpion Boxing Milano</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>393514088140</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+34635541239</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>kickbarcelona@gmail.com</t>
+          <t>Conversation existed on old number</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>@kickbarcelona</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM + email + WA sent (email re-co</t>
+          <t>REPLIED before - re-contact first</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>L074</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Lucero Muay Thai Madrid</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>34633215305</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Conversation existed on old number</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>REPLIED before - re-contact first</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Lead ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>IG Handle</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>L001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Golden Kyu Barcelona</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>+34670425918</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>info@goldenkyu.com</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>@goldenkyu_bcn</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>L002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kick Barcelona</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>+34635541239</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>kickbarcelona@gmail.com</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>@kickbarcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>L003</t>
         </is>
       </c>
@@ -559,14 +707,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>+34620953033</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>+34620953033</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>hola@warriorsbarcelona.com</t>
@@ -575,1242 +723,1938 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>@warriorsbarcelona</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>COMPLETE: already-following + IG DM + email + WA sent (email</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>L007</t>
+          <t>L020</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Invicta Martial Arts</t>
+          <t>Ippon Gear España</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>34611612163</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>351910479457</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>info@invictamaa.com</t>
+          <t>info@ippongear.es</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>@invictamaa</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=ok dm=sent email=sent wa={"ok":true,"last":</t>
+          <t>@ippongear_spain</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>L020</t>
+          <t>L021</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ippon Gear España</t>
+          <t>Splinters Jiu-Jitsu &amp; MMA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>34622212369</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>34611612163</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>info@ippongear.es</t>
+          <t>splintersmadrid@gmail.com</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>@ippongear_spain</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=ok dm=sent email=sent wa={"ok":true,"last":</t>
+          <t>@splintersmadrid</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>L021</t>
+          <t>L023</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Splinters Jiu-Jitsu &amp; MMA</t>
+          <t>Al-Andalus Judo Sevilla</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>34625621710</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>34622212369</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>splintersmadrid@gmail.com</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>@splintersmadrid</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM sent</t>
-        </is>
-      </c>
+          <t>info@judosevilla.com</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L023</t>
+          <t>L024</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Al-Andalus Judo Sevilla</t>
+          <t>KALMMA Fight Club</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>34699506391</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>34625621710</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>info@judosevilla.com</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last</t>
+          <t>info@kalmmafightclub.com</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>@kalmmafightclub</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>L024</t>
+          <t>L025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>KALMMA Fight Club</t>
+          <t>Judo Kitaro</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>34649036805</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>34699506391</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>info@kalmmafightclub.com</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>@kalmmafightclub</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG DM sent (follow btn n/a - already following)</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>L025</t>
+          <t>L026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Judo Kitaro</t>
+          <t>Brazilian Fight Lisboa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>351910349061</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>34649036805</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last</t>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>brazilian.fight.lisboa@gmail.com</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>@brazilian.fight.lisboa</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>L026</t>
+          <t>L027</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Brazilian Fight Lisboa</t>
+          <t>K.O. Team Portugal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>351963919855</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>351910349061</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>brazilian.fight.lisboa@gmail.com</t>
+          <t>info@koteam.pt</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>@brazilian.fight.lisboa</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=sent wa={"ok":true,"la</t>
+          <t>@koteamportugal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>L027</t>
+          <t>L028</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>K.O. Team Portugal</t>
+          <t>Team Duramuk</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>351967734557</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>351963919855</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>info@koteam.pt</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>@koteamportugal</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM sent + email sent (info@koteam</t>
+          <t>@team.duramuk</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>L028</t>
+          <t>L029</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Team Duramuk</t>
+          <t>Five Elements Academy Jiu-Jitsu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
+          <t>351915267080</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
           <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>351967734557</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>@team.duramuk</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM + WA sent (no public email - W</t>
+          <t>@fiveelementsjiujitsu</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>L029</t>
+          <t>L030</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Five Elements Academy Jiu-Jitsu</t>
+          <t>Gracie Lisboa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
+          <t>351967599340</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>351915267080</t>
-        </is>
-      </c>
       <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>@fiveelementsjiujitsu</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>COMPLETE: IG followed + IG DM sent</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>L030</t>
+          <t>L031</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gracie Lisboa</t>
+          <t>APKO Okinawa Karate</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>351961320560</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>351967599340</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>apko.geral@gmail.com</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>L031</t>
+          <t>L054</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>APKO Okinawa Karate</t>
+          <t>FullGym 24h Vilafranca</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>34621413059</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>351961320560</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>apko.geral@gmail.com</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last</t>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>@fullgymvilafranca</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>L054</t>
+          <t>L132</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FullGym 24h Vilafranca</t>
+          <t>Alvaro Campeao</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>351916033601</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34621413059</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>pt.alvarocampeao@gmail.com</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>@fullgymvilafranca</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=ok dm=sent email=None wa={"ok":true,"last":</t>
+          <t>@alvarotdcampeao</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>L132</t>
+          <t>L140</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Alvaro Campeao</t>
+          <t>Fight Center Boxing</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>33783401554</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>351916033601</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>pt.alvarocampeao@gmail.com</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>@alvarotdcampeao</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent + IG followed + IG DM sent (phone NOT o</t>
-        </is>
-      </c>
+          <t>fightboxing13@gmail.com</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>L140</t>
+          <t>L144</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fight Center Boxing</t>
+          <t>Angels Boxing</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>353873256588</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33783401554</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>fightboxing13@gmail.com</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent (phone NOT on WhatsApp — verified)</t>
+          <t>byrnereg43@gmail.com</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>@coach_reg.byrne</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>L144</t>
+          <t>L153</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Angels Boxing</t>
+          <t>Bomaye Gym München</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>491737513627</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>353873256588</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>byrnereg43@gmail.com</t>
-        </is>
-      </c>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>@coach_reg.byrne</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=recipient-not-register</t>
+          <t>@bomayegym_munich</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>L153</t>
+          <t>L154</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bomaye Gym München</t>
+          <t>Martial Arts Center München</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>491708890687</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>491737513627</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>@bomayegym_munich</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=clicked dm=sent email=None wa=no-composer</t>
-        </is>
-      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>info@ving-tsun.net</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>L154</t>
+          <t>L158</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Martial Arts Center München</t>
+          <t>Crossbox Gym</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>34649316067</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>491708890687</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>info@ving-tsun.net</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa=no-composer</t>
+          <t>crossboxgym@protonmail.com</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>@crossboxgym</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>L158</t>
+          <t>L159</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Crossbox Gym</t>
+          <t>Ali Promotions BCN</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>34687075304</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>34649316067</t>
-        </is>
-      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>crossboxgym@protonmail.com</t>
+          <t>alipromotions.bcn@gmail.com</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>@crossboxgym</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=sent wa=no-composer</t>
+          <t>@alipromotions.bcn</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>L159</t>
+          <t>L160</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ali Promotions BCN</t>
+          <t>Hybrd Academy</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
+          <t>34692382544</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>34687075304</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>alipromotions.bcn@gmail.com</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>@alipromotions.bcn</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=clicked dm=sent email=sent wa=no-composer</t>
-        </is>
-      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>L160</t>
+          <t>L177</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Hybrd Academy</t>
+          <t>Academiamariopadilla</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
+          <t>34659425174</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>34692382544</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>mario@academiamariopadilla.com</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>COMPLETE: follow=None dm=None email=None wa=no-composer</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>L177</t>
+          <t>L183</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Academiamariopadilla</t>
+          <t>Shudokan</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
+          <t>34661571463</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>34659425174</t>
-        </is>
-      </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>mario@academiamariopadilla.com</t>
+          <t>info@shudokan.es</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>@ancora_themes</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@shudokan.roje</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>L183</t>
+          <t>L185</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Shudokan</t>
+          <t>Clubtakeda</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
+          <t>34620517614</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>34661571463</t>
-        </is>
-      </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>info@shudokan.es</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>@shudokan.roje</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
-        </is>
-      </c>
+          <t>info.clubtakeda@gmail.com</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>L185</t>
+          <t>L187</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Clubtakeda</t>
+          <t>Crossboxgym</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
+          <t>34649316067</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>34620517614</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>info.clubtakeda@gmail.com</t>
+          <t>crossboxgym@gmail.com</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>L187</t>
+          <t>L188</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Crossboxgym</t>
+          <t>Crossboxing</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
+          <t>34620067869</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>34649316067</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>crossboxgym@gmail.com</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>info@crossboxing.com</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>@crossboxing.es</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>L188</t>
+          <t>L252</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Crossboxing</t>
+          <t>Dgmma</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>491773216092</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>34620067869</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>info@crossboxing.com</t>
+          <t>hello@dgmma.de</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>@crossboxing.es</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@dragongatemma</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>L252</t>
+          <t>L254</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dgmma</t>
+          <t>Elysium Mma</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
+          <t>4917643525310</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>491773216092</t>
-        </is>
-      </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>hello@dgmma.de</t>
+          <t>info@elysium-mma.de</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>@dragongatemma</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@elysium_mma_munich</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>L254</t>
+          <t>L255</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Elysium Mma</t>
+          <t>Tripleonegym</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
+          <t>491734496111</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>4917643525310</t>
-        </is>
-      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>info@elysium-mma.de</t>
+          <t>info@tripleonegym.de</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>@elysium_mma_munich</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@tripleonegym</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>L255</t>
+          <t>L267</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Tripleonegym</t>
+          <t>Kickboxingvomero</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>39335344423</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>491734496111</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>info@tripleonegym.de</t>
+          <t>kickboxingvomero@gmail.com</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>@tripleonegym</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@kickboxingvomero</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>L267</t>
+          <t>L269</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Kickboxingvomero</t>
+          <t>Mgmboxeisland</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
+          <t>393896699615</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>39335344423</t>
-        </is>
-      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>kickboxingvomero@gmail.com</t>
+          <t>info@101sport.net</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>@kickboxingvomero</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@MGM_MIlano</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>L269</t>
+          <t>L287</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mgmboxeisland</t>
+          <t>Bokshuis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>31642692144</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>393896699615</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>info@101sport.net</t>
+          <t>info@bokshuis.nl</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>@MGM_MIlano</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@bokshuis</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>L287</t>
+          <t>L347</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bokshuis</t>
+          <t>Tkoboxingclub</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>447538916121</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>31642692144</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>info@bokshuis.nl</t>
+          <t>team@tkoboxingclub.co.uk</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>@bokshuis</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@tkoboxingclub</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>L347</t>
+          <t>L350</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Tkoboxingclub</t>
+          <t>Kenglengmuaythai</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
+          <t>07496652323</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>447538916121</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>team@tkoboxingclub.co.uk</t>
+          <t>kenglengmuaythai@gmail.com</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>@tkoboxingclub</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+          <t>@kengleng.muaythai</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>L350</t>
+          <t>L354</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Kenglengmuaythai</t>
+          <t>Adrenalinemt</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
+          <t>447920887358</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>07496652323</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>kenglengmuaythai@gmail.com</t>
+          <t>admin@adrenalinemt.uk</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>@kengleng.muaythai</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>L354</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Adrenalinemt</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
+          <t>@adrenaline_muay_thai</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Lead ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Country</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Old status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>L039</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kick &amp; Punch Milano DownTown</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>393914124452</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG followed + IG DM sent + WhatsApp sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>L044</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Sokudo Gym Hoorn</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>31229215582</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG followed + IG DM sent + WhatsApp sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>L046</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Gracie Barra Braga</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>351927773854</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG DM sent + WhatsApp sent (follow btn n</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L048</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kickboxing Madrid</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>34685660511</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG follow=ok + DM sent + WhatsApp sent +</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>L049</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CrossBox Gym</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>34649316067</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG follow=ok + DM sent + WhatsApp sent +</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>L050</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DM Fight</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>34613268619</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG follow=ok + DM sent + WhatsApp sent +</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>L051</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Draco Fight Club</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>34667720380</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>COMPLETE: IG follow=ok + DM sent + WhatsApp sent +</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>L055</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Slava Legacy Gym</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>34674387362</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent (email n/a) + IG follow pe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>L056</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wuxing Madrid</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>34643340522</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG follow p</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>L059</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Mugendo Martial Arts Eixample</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>34646739122</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent (Mugendo Eixample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L062</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HardiFit</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>34662494150</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + IG followed + IG DM sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L065</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Fight Culture</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>351963631744</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + IG followed + IG DM sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L066</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Porradaria Ate'o Talho</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>351913200732</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent (Porradaria)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>L068</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Lucero Muay Thai Madrid</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>34633215305</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent (Lucero)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>L072</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Muay Thai Kassel</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>4956181696280</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + IG followed + IG DM sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>L090</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Akhi Sport Gym</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>31650514751</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>L093</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Amsterdam Training Center</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>31627006861</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>L094</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Freddy's Kickboxing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>31613701879</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L096</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Sukhothai Academy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4978219228338</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>L097</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KOI Gym Frankfurt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>491743505229</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>L098</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Champs Kickboxing Berlin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>4930233208320</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>L106</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Boxing Trainer London</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>447790210031</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
         <is>
           <t>UK</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>447920887358</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>admin@adrenalinemt.uk</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>@adrenaline_muay_thai</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>COMPLETE: email sent</t>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>L130</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PT do Bairro</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>351931468801</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>L134</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Studio Absoluto JJ</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>351934624841</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>L135</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AMDKP</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>351911165714</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>L138</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Spirit Academy 74</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>41796061009</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>L139</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Beat 35 Studio</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>33672587591</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>L141</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Le Hook Vieux Lille</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>33766685436</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + IG followed + IG DM sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>L142</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bennies Boxing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>447961557534</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>L163</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Armazém Jiu-Jitsu</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>351925896645</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>L164</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Fred Motta Muay Thai</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>351968718777</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>L165</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Z Fortes Muay Thai</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>351965577023</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>COMPLETE: WhatsApp sent + email sent + IG followed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Day 8 catch-up: hunt + pipeline after 20:00 UTC session died early (0 leads hunted then)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -511,7 +511,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>COMPLETE: IG followed + IG DM + WA + email sent</t>
+          <t>COMPLETE: IG followed + IG DM + WA + email sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>COMPLETE: IG followed + IG DM + email + WA sent (email re-confirmed v4)</t>
+          <t>COMPLETE: IG followed + IG DM + email + WA sent (email re-confirmed v4) | COMPLETE: email sent (Day 6, 2026-10-19)</t>
         </is>
       </c>
       <c r="H3" t="inlineStr"/>
@@ -591,7 +591,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>COMPLETE: already-following + IG DM + email + WA sent (email re-confirmed v4)</t>
+          <t>COMPLETE: already-following + IG DM + email + WA sent (email re-confirmed v4) | COMPLETE: email sent (Day 6, 2026-10-19)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Follow-up sent 2026-10-16 (reference old pads+gloves chat + free logo branding value). Awaiting reply.</t>
+          <t xml:space="preserve"> | Follow-up 2 sent 2026-10-17 (training vs competition question). | COMPLETE: email sent (Day 6, 2026-10-19) | WA sent (Day 6) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=ok dm=sent email=sent wa={"ok":true,"last":["Hola Ippon Gear España! \n\n\n\nHola Ippon G"]}</t>
+          <t>COMPLETE: follow=ok dm=sent email=sent wa={"ok":true,"last":["Hola Ippon Gear España! \n\n\n\nHola Ippon G"]} | COMPLETE: email sent (Day 6, 2026-10-19) | WA sent (Day 6) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>COMPLETE: IG followed + IG DM sent | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: IG followed + IG DM sent | WA sent (Day 5 wave) | COMPLETE: email sent (Day 6, 2026-10-19)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -751,7 +751,7 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last":["Hola Al-Andalus Judo Sevilla! \n\n\n\nwe mak"]}</t>
+          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last":["Hola Al-Andalus Judo Sevilla! \n\n\n\nwe mak"]} | COMPLETE: email sent (Day 6, 2026-10-19) | WA sent (Day 6)</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>COMPLETE: IG DM sent (follow btn n/a - already following) | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: IG DM sent (follow btn n/a - already following) | WA sent (Day 5 wave) | COMPLETE: email sent (Day 6, 2026-10-19)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -827,7 +827,7 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last":["Hola Judo Kitaro! \n\n\n\nwe make custom mar"]}</t>
+          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last":["Hola Judo Kitaro! \n\n\n\nwe make custom mar"]} | WA sent (Day 6)</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=sent wa={"ok":true,"last":["Hola Brazilian Fight Lisboa! \n\n\n\nwe make"]}</t>
+          <t xml:space="preserve"> | REPLIED + PT follow-up sent 2026-10-20 (quantity question, factory prices, academy branding). | IG not found</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1021,7 +1021,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last":["Hola Gracie Lisboa! \n\n\n\nmartial arts &amp; s"]}</t>
+          <t>COMPLETE: follow=None dm=None email=None wa={"ok":true,"last":["Hola Gracie Lisboa! \n\n\n\nmartial arts &amp; s"]} | WA sent (Day 6)</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1059,7 +1059,7 @@
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last":["Hola APKO Okinawa Karate! \n\n\n\nmartial ar"]}</t>
+          <t>COMPLETE: follow=None dm=None email=sent wa={"ok":true,"last":["Hola APKO Okinawa Karate! \n\n\n\nmartial ar"]} | COMPLETE: email sent (Day 6, 2026-10-19) | WA sent (Day 6)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1086,7 +1086,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34621413059</t>
+          <t>+34621413059</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=ok dm=sent email=None wa={"ok":true,"last":["Hello FullGym 24h Vilafranca! \n\n\n\nwe pro"]}</t>
+          <t>COMPLETE: follow=ok dm=sent email=None wa={"ok":true,"last":["Hello FullGym 24h Vilafranca! \n\n\n\nwe pro"]} | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>33664204654</t>
+          <t>+33664204654</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Follow-up sent 2026-10-16 (fight-team package angle: 2-3 items + exact pricing offer). Awaiting reply.</t>
+          <t xml:space="preserve"> | Follow-up 2 sent 2026-10-17 (default 10x package quote offer). | COMPLETE: email sent (Day 6, 2026-10-19) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1166,7 +1166,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>393514088140</t>
+          <t>+393514088140</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Follow-up sent 2026-10-16 (ultra-short + 'reply yes' micro-commitment). Awaiting reply.</t>
+          <t xml:space="preserve"> | Follow-up 2 sent 2026-10-17 (EUR 19.50 anchor + no-minimum trial offer). | COMPLETE: email sent (Day 6, 2026-10-19) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>351916033601</t>
+          <t>+351916033601</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>HOT LEAD (payment stage): asked Dirham or Euro. Answered: Euro pricing, he pays Dirham via Western Union, we receive local currency. Awaiting his confirmation + logo. Sample EUR 77.40.</t>
+          <t xml:space="preserve"> | Follow-up 2 sent 2026-10-17 (mockup-first offer, EUR 77.40 all-in). Awaiting logo. | COMPLETE: email sent (Day 6, 2026-10-19) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>33783401554</t>
+          <t>+33783401554</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>353873256588</t>
+          <t>+353873256588</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1303,7 +1303,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=recipient-not-registered wa={"ok":true,"last":["Hello Angels Boxing! \n\n\n\nmartial arts &amp; "]}</t>
+          <t>COMPLETE: follow=no-btn dm=sent email=recipient-not-registered wa={"ok":true,"last":["Hello Angels Boxing! \n\n\n\nmartial arts &amp; "]} | EMAIL FAILED (Day 6) | IG follow=no-btn dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>491737513627</t>
+          <t>+491737513627</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=clicked dm=sent email=None wa=no-composer</t>
+          <t>COMPLETE: follow=clicked dm=sent email=None wa=no-composer | IG follow=ok dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>491708890687</t>
+          <t>+491708890687</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1379,7 +1379,7 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=sent wa=no-composer</t>
+          <t>COMPLETE: follow=None dm=None email=sent wa=no-composer | COMPLETE: email sent (Day 6, 2026-10-19)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1391,12 +1391,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>L158</t>
+          <t>L159</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Crossbox Gym</t>
+          <t>Ali Promotions BCN</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1406,22 +1406,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>34649316067</t>
+          <t>+34687075304</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>crossboxgym@protonmail.com</t>
+          <t>alipromotions.bcn@gmail.com</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>@crossboxgym</t>
+          <t>@alipromotions.bcn</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=no-btn dm=sent email=sent wa=no-composer</t>
+          <t>COMPLETE: follow=clicked dm=sent email=sent wa=no-composer | COMPLETE: email sent (Day 6, 2026-10-19) | IG follow=ok dm=sent (Day 6)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1433,12 +1433,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>L159</t>
+          <t>L160</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ali Promotions BCN</t>
+          <t>Hybrd Academy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1448,22 +1448,14 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>34687075304</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>alipromotions.bcn@gmail.com</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>@alipromotions.bcn</t>
-        </is>
-      </c>
+          <t>+34692382544</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=clicked dm=sent email=sent wa=no-composer</t>
+          <t>COMPLETE: follow=None dm=None email=None wa=no-composer</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1475,12 +1467,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>L160</t>
+          <t>L177</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hybrd Academy</t>
+          <t>Academiamariopadilla</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1490,31 +1482,35 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>34692382544</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
+          <t>34659425174</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>mario@academiamariopadilla.com</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>COMPLETE: follow=None dm=None email=None wa=no-composer</t>
+          <t>COMPLETE: email sent [IG handle was junk - removed] | WA sent (Day 5 wave)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Day 3 hunt batch</t>
+          <t>Day 4 night batch</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>L177</t>
+          <t>L183</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Academiamariopadilla</t>
+          <t>Shudokan</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1524,18 +1520,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>34659425174</t>
+          <t>34661571463</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>mario@academiamariopadilla.com</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>info@shudokan.es</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>@shudokan.roje</t>
+        </is>
+      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent [IG handle was junk - removed] | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 5 wave)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1547,12 +1547,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>L183</t>
+          <t>L185</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Shudokan</t>
+          <t>Clubtakeda</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1562,22 +1562,18 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>34661571463</t>
+          <t>34620517614</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>info@shudokan.es</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>@shudokan.roje</t>
-        </is>
-      </c>
+          <t>info.clubtakeda@gmail.com</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: email sent | WA sent (Day 5 wave)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1589,12 +1585,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>L185</t>
+          <t>L187</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Clubtakeda</t>
+          <t>Crossboxgym</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1604,12 +1600,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>34620517614</t>
+          <t>34649316067</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>info.clubtakeda@gmail.com</t>
+          <t>crossboxgym@gmail.com</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -1627,12 +1623,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>L187</t>
+          <t>L188</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Crossboxgym</t>
+          <t>Crossboxing</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1642,18 +1638,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>34649316067</t>
+          <t>34620067869</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>crossboxgym@gmail.com</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>info@crossboxing.com</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>@crossboxing.es</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: email sent | IG profile not found | IG profile not found | IG profile not found | IG profile not found | IG profile not found | WA sent (Day 5 wave) | IG not found</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1665,37 +1665,37 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>L188</t>
+          <t>L252</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Crossboxing</t>
+          <t>Dgmma</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>34620067869</t>
+          <t>491773216092</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>info@crossboxing.com</t>
+          <t>hello@dgmma.de</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>@crossboxing.es</t>
+          <t>@dragongatemma</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG profile not found | IG profile not found | IG profile not found | IG profile not found | IG profile not found | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 5 wave)</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1707,12 +1707,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>L252</t>
+          <t>L254</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Dgmma</t>
+          <t>Elysium Mma</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1722,22 +1722,22 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>491773216092</t>
+          <t>+4917643525310</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>hello@dgmma.de</t>
+          <t>info@elysium-mma.de</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>@dragongatemma</t>
+          <t>@elysium_mma_munich</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 5 wave)</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1749,12 +1749,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>L254</t>
+          <t>L255</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Elysium Mma</t>
+          <t>Tripleonegym</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1764,22 +1764,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>4917643525310</t>
+          <t>+491734496111</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>info@elysium-mma.de</t>
+          <t>info@tripleonegym.de</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>@elysium_mma_munich</t>
+          <t>@tripleonegym</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA FAILED (Day 7): no-composer</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -1791,37 +1791,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>L255</t>
+          <t>L267</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tripleonegym</t>
+          <t>Kickboxingvomero</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>491734496111</t>
+          <t>+39335344423</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>info@tripleonegym.de</t>
+          <t>kickboxingvomero@gmail.com</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>@tripleonegym</t>
+          <t>@kickboxingvomero</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -1833,12 +1833,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>L267</t>
+          <t>L269</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Kickboxingvomero</t>
+          <t>Mgmboxeisland</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1848,22 +1848,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>39335344423</t>
+          <t>+393896699615</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>kickboxingvomero@gmail.com</t>
+          <t>info@101sport.net</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>@kickboxingvomero</t>
+          <t>@MGM_MIlano</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1875,37 +1875,37 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>L269</t>
+          <t>L287</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Mgmboxeisland</t>
+          <t>Bokshuis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>393896699615</t>
+          <t>+31642692144</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>info@101sport.net</t>
+          <t>info@bokshuis.nl</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>@MGM_MIlano</t>
+          <t>@bokshuis</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=ok dm=sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -1917,37 +1917,37 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>L287</t>
+          <t>L347</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bokshuis</t>
+          <t>Tkoboxingclub</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>31642692144</t>
+          <t>+447538916121</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>info@bokshuis.nl</t>
+          <t>team@tkoboxingclub.co.uk</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>@bokshuis</t>
+          <t>@tkoboxingclub</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=ok dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=clicked dm=sent | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -1959,12 +1959,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>L347</t>
+          <t>L350</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Tkoboxingclub</t>
+          <t>Kenglengmuaythai</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1974,17 +1974,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>447538916121</t>
+          <t>+07496652323</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>team@tkoboxingclub.co.uk</t>
+          <t>kenglengmuaythai@gmail.com</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>@tkoboxingclub</t>
+          <t>@kengleng.muaythai</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2001,12 +2001,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>L350</t>
+          <t>L354</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Kenglengmuaythai</t>
+          <t>Adrenalinemt</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2016,22 +2016,22 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>07496652323</t>
+          <t>+447920887358</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>kenglengmuaythai@gmail.com</t>
+          <t>admin@adrenalinemt.uk</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>@kengleng.muaythai</t>
+          <t>@adrenaline_muay_thai</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=clicked dm=sent</t>
+          <t>COMPLETE: email sent | IG follow=clicked dm=sent | WA sent (Day 8) - verified transcript</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2043,42 +2043,110 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>L354</t>
+          <t>L581</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Adrenalinemt</t>
+          <t>Pugilistica Elite Milano</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>447920887358</t>
+          <t>+393514002388</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>admin@adrenalinemt.uk</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>@adrenaline_muay_thai</t>
-        </is>
-      </c>
+          <t>info@pugilisticaelite.com</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG follow=clicked dm=sent</t>
+          <t>COMPLETE: email sent (Day 7 test-send, 2026-10-19) | WA sent (Day 7) - verified transcript</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Day 4 night batch</t>
+          <t>Hunted 2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>L585</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Fight District Amsterdam</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>+31629144029</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>hello@fightdistrict.nl</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>HUNTED (Day 6 pre-dawn, schema repaired Day 7) | COMPLETE: email sent (Day 7, 2026-10-19) | WA sent (Day 7) - verified transcript</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Hunted 2026-10-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>L595</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Combatgym.ch</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>+41792740620</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>HUNTED (Day 6 pre-dawn, schema repaired Day 7) | WA sent (Day 7) - verified transcript</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Hunted 2026-10-19 1AM</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bounce cleanup: 35 bounced-email leads marked FAILED, 13 scrape-contaminated email rows excluded (2026-10-24)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -1653,7 +1653,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>COMPLETE: email sent | IG profile not found | IG profile not found | IG profile not found | IG profile not found | IG profile not found | WA sent (Day 5 wave) | IG not found</t>
+          <t>COMPLETE: email sent | IG profile not found | IG profile not found | IG profile not found | IG profile not found | IG profile not found | WA sent (Day 5 wave) | IG not found | EMAIL FAILED (bounce confirmed 2026-10-24)</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2823,7 +2823,7 @@
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-21) | WA sent (Day 8 manual wave, 2026-10-21) | COMPLETE: email sent (Daily 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-21) | WA sent (Day 8 manual wave, 2026-10-21) | COMPLETE: email sent (Daily 2026-10-23) | EMAIL FAILED (bounce confirmed 2026-10-24)</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
@@ -5773,7 +5773,7 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-21) | COMPLETE: email sent (sprint Day 1, 2026-10-22)</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-21) | COMPLETE: email sent (sprint Day 1, 2026-10-22) | EMAIL FAILED (bounce confirmed 2026-10-24) | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H155" t="inlineStr"/>
@@ -9713,7 +9713,7 @@
       <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: garbage scraped email</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: garbage scraped email | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H279" t="inlineStr"/>
@@ -15277,7 +15277,7 @@
       <c r="F449" t="inlineStr"/>
       <c r="G449" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H449" t="inlineStr"/>
@@ -15345,7 +15345,7 @@
       <c r="F451" t="inlineStr"/>
       <c r="G451" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H451" t="inlineStr"/>
@@ -15413,7 +15413,7 @@
       <c r="F453" t="inlineStr"/>
       <c r="G453" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED: image-filename scraped as email | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H453" t="inlineStr"/>
@@ -16325,7 +16325,7 @@
       <c r="F481" t="inlineStr"/>
       <c r="G481" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t xml:space="preserve">HUNTED (gmaps 2PM 2026-10-23) | EXCLUDED (scrape contamination: email cell is not a valid address) </t>
         </is>
       </c>
       <c r="H481" t="inlineStr"/>

</xml_diff>

<commit_message>
Day-11 final: +4 IG follow+DM (Lisbon/Zurich), tracker + WA list rebuilt (1930 leads)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -29423,7 +29423,7 @@
       </c>
       <c r="G890" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | IG profile not found (2026-10-25)</t>
         </is>
       </c>
       <c r="H890" t="inlineStr"/>
@@ -31207,7 +31207,7 @@
       </c>
       <c r="G946" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | IG follow=ok dm=sent (Daily 2026-10-25)</t>
         </is>
       </c>
       <c r="H946" t="inlineStr"/>
@@ -31827,7 +31827,7 @@
       </c>
       <c r="G966" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | IG follow=ok dm=sent (Daily 2026-10-25)</t>
         </is>
       </c>
       <c r="H966" t="inlineStr"/>

</xml_diff>

<commit_message>
day12 outreach 2026-10-26 (email wave + IG pass + tracker)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1057"/>
+  <dimension ref="A1:H1074"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -11473,7 +11473,7 @@
       <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H333" t="inlineStr"/>
@@ -11635,7 +11635,7 @@
       <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H338" t="inlineStr"/>
@@ -11703,7 +11703,7 @@
       <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H340" t="inlineStr"/>
@@ -11737,7 +11737,7 @@
       <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H341" t="inlineStr"/>
@@ -11801,7 +11801,7 @@
       <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H343" t="inlineStr"/>
@@ -12031,7 +12031,7 @@
       <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H350" t="inlineStr"/>
@@ -12585,7 +12585,7 @@
       <c r="F367" t="inlineStr"/>
       <c r="G367" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H367" t="inlineStr"/>
@@ -12683,7 +12683,7 @@
       <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H370" t="inlineStr"/>
@@ -12883,7 +12883,7 @@
       <c r="F376" t="inlineStr"/>
       <c r="G376" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H376" t="inlineStr"/>
@@ -13101,7 +13101,7 @@
       <c r="F383" t="inlineStr"/>
       <c r="G383" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H383" t="inlineStr"/>
@@ -13361,7 +13361,7 @@
       <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H391" t="inlineStr"/>
@@ -13459,7 +13459,7 @@
       <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H394" t="inlineStr"/>
@@ -13655,7 +13655,7 @@
       <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H400" t="inlineStr"/>
@@ -13889,7 +13889,7 @@
       <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H407" t="inlineStr"/>
@@ -14051,7 +14051,7 @@
       <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H412" t="inlineStr"/>
@@ -14085,7 +14085,7 @@
       <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H413" t="inlineStr"/>
@@ -14119,7 +14119,7 @@
       <c r="F414" t="inlineStr"/>
       <c r="G414" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H414" t="inlineStr"/>
@@ -14153,7 +14153,7 @@
       <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H415" t="inlineStr"/>
@@ -29137,7 +29137,7 @@
       <c r="F881" t="inlineStr"/>
       <c r="G881" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H881" t="inlineStr"/>
@@ -29231,7 +29231,7 @@
       <c r="F884" t="inlineStr"/>
       <c r="G884" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (day12 QA: email not verifiable on the lead own site)</t>
         </is>
       </c>
       <c r="H884" t="inlineStr"/>
@@ -29259,13 +29259,13 @@
       </c>
       <c r="E885" t="inlineStr">
         <is>
-          <t>sdbenfica@vma.com.pt, alfragide@vma.com.pt, email@dominio.pt</t>
+          <t>sdbenfica@vma.com.pt</t>
         </is>
       </c>
       <c r="F885" t="inlineStr"/>
       <c r="G885" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; sdbenfica@vma.com.pt; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H885" t="inlineStr"/>
@@ -29329,7 +29329,7 @@
       <c r="F887" t="inlineStr"/>
       <c r="G887" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H887" t="inlineStr"/>
@@ -29547,7 +29547,7 @@
       <c r="F894" t="inlineStr"/>
       <c r="G894" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H894" t="inlineStr"/>
@@ -29729,13 +29729,13 @@
       </c>
       <c r="E900" t="inlineStr">
         <is>
-          <t>info@anks.pt, u003einfo@anks.pt</t>
+          <t>info@anks.pt</t>
         </is>
       </c>
       <c r="F900" t="inlineStr"/>
       <c r="G900" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@anks.pt; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H900" t="inlineStr"/>
@@ -29799,7 +29799,7 @@
       <c r="F902" t="inlineStr"/>
       <c r="G902" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H902" t="inlineStr"/>
@@ -29827,13 +29827,13 @@
       </c>
       <c r="E903" t="inlineStr">
         <is>
-          <t>hussainmazhar558@gmail.com, info@tehreembco.com</t>
+          <t>info@tehreembco.com</t>
         </is>
       </c>
       <c r="F903" t="inlineStr"/>
       <c r="G903" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@tehreembco.com; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H903" t="inlineStr"/>
@@ -29957,7 +29957,7 @@
       <c r="F907" t="inlineStr"/>
       <c r="G907" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H907" t="inlineStr"/>
@@ -30055,7 +30055,7 @@
       <c r="F910" t="inlineStr"/>
       <c r="G910" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H910" t="inlineStr"/>
@@ -30183,7 +30183,7 @@
       <c r="F914" t="inlineStr"/>
       <c r="G914" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H914" t="inlineStr"/>
@@ -30277,7 +30277,7 @@
       <c r="F917" t="inlineStr"/>
       <c r="G917" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H917" t="inlineStr"/>
@@ -30533,7 +30533,7 @@
       <c r="F925" t="inlineStr"/>
       <c r="G925" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H925" t="inlineStr"/>
@@ -30597,7 +30597,7 @@
       <c r="F927" t="inlineStr"/>
       <c r="G927" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H927" t="inlineStr"/>
@@ -30631,7 +30631,7 @@
       <c r="F928" t="inlineStr"/>
       <c r="G928" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H928" t="inlineStr"/>
@@ -30665,7 +30665,7 @@
       <c r="F929" t="inlineStr"/>
       <c r="G929" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H929" t="inlineStr"/>
@@ -30699,7 +30699,7 @@
       <c r="F930" t="inlineStr"/>
       <c r="G930" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H930" t="inlineStr"/>
@@ -30733,7 +30733,7 @@
       <c r="F931" t="inlineStr"/>
       <c r="G931" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H931" t="inlineStr"/>
@@ -30891,7 +30891,7 @@
       <c r="F936" t="inlineStr"/>
       <c r="G936" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H936" t="inlineStr"/>
@@ -30955,7 +30955,7 @@
       <c r="F938" t="inlineStr"/>
       <c r="G938" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H938" t="inlineStr"/>
@@ -31113,7 +31113,7 @@
       <c r="F943" t="inlineStr"/>
       <c r="G943" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H943" t="inlineStr"/>
@@ -31425,7 +31425,7 @@
       <c r="F953" t="inlineStr"/>
       <c r="G953" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H953" t="inlineStr"/>
@@ -31759,7 +31759,7 @@
       <c r="F964" t="inlineStr"/>
       <c r="G964" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H964" t="inlineStr"/>
@@ -31787,13 +31787,13 @@
       </c>
       <c r="E965" t="inlineStr">
         <is>
-          <t>contacto@saitamabjj.com, jane@framer.com</t>
+          <t>contacto@saitamabjj.com</t>
         </is>
       </c>
       <c r="F965" t="inlineStr"/>
       <c r="G965" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; contacto@saitamabjj.com; name/site slug match) | EXCLUDED (day12 QA: email not verifiable on the lead own site)</t>
         </is>
       </c>
       <c r="H965" t="inlineStr"/>
@@ -31921,7 +31921,7 @@
       <c r="F969" t="inlineStr"/>
       <c r="G969" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H969" t="inlineStr"/>
@@ -32015,7 +32015,7 @@
       <c r="F972" t="inlineStr"/>
       <c r="G972" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H972" t="inlineStr"/>
@@ -32049,7 +32049,7 @@
       <c r="F973" t="inlineStr"/>
       <c r="G973" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H973" t="inlineStr"/>
@@ -32083,7 +32083,7 @@
       <c r="F974" t="inlineStr"/>
       <c r="G974" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H974" t="inlineStr"/>
@@ -32111,13 +32111,13 @@
       </c>
       <c r="E975" t="inlineStr">
         <is>
-          <t>center@taekwondo-terranova.com, m.delena@taekwondo-zuerich.ch</t>
+          <t>center@taekwondo-terranova.com</t>
         </is>
       </c>
       <c r="F975" t="inlineStr"/>
       <c r="G975" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; center@taekwondo-terranova.com; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H975" t="inlineStr"/>
@@ -32151,7 +32151,7 @@
       <c r="F976" t="inlineStr"/>
       <c r="G976" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H976" t="inlineStr"/>
@@ -32185,7 +32185,7 @@
       <c r="F977" t="inlineStr"/>
       <c r="G977" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H977" t="inlineStr"/>
@@ -32219,7 +32219,7 @@
       <c r="F978" t="inlineStr"/>
       <c r="G978" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H978" t="inlineStr"/>
@@ -32313,7 +32313,7 @@
       <c r="F981" t="inlineStr"/>
       <c r="G981" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H981" t="inlineStr"/>
@@ -32381,7 +32381,7 @@
       <c r="F983" t="inlineStr"/>
       <c r="G983" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H983" t="inlineStr"/>
@@ -32445,7 +32445,7 @@
       <c r="F985" t="inlineStr"/>
       <c r="G985" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H985" t="inlineStr"/>
@@ -32543,7 +32543,7 @@
       <c r="F988" t="inlineStr"/>
       <c r="G988" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H988" t="inlineStr"/>
@@ -32637,7 +32637,7 @@
       <c r="F991" t="inlineStr"/>
       <c r="G991" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H991" t="inlineStr"/>
@@ -32701,7 +32701,7 @@
       <c r="F993" t="inlineStr"/>
       <c r="G993" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H993" t="inlineStr"/>
@@ -32765,7 +32765,7 @@
       <c r="F995" t="inlineStr"/>
       <c r="G995" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H995" t="inlineStr"/>
@@ -32829,7 +32829,7 @@
       <c r="F997" t="inlineStr"/>
       <c r="G997" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H997" t="inlineStr"/>
@@ -33017,7 +33017,7 @@
       <c r="F1003" t="inlineStr"/>
       <c r="G1003" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1003" t="inlineStr"/>
@@ -33051,7 +33051,7 @@
       <c r="F1004" t="inlineStr"/>
       <c r="G1004" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1004" t="inlineStr"/>
@@ -33173,13 +33173,13 @@
       </c>
       <c r="E1008" t="inlineStr">
         <is>
-          <t>info@swisskarate.ch, wallisellen@swisskarate.ch</t>
+          <t>info@swisskarate.ch</t>
         </is>
       </c>
       <c r="F1008" t="inlineStr"/>
       <c r="G1008" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@swisskarate.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1008" t="inlineStr"/>
@@ -33207,13 +33207,13 @@
       </c>
       <c r="E1009" t="inlineStr">
         <is>
-          <t>user@domain.com, info@meintempel.ch</t>
+          <t>info@meintempel.ch</t>
         </is>
       </c>
       <c r="F1009" t="inlineStr"/>
       <c r="G1009" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@meintempel.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1009" t="inlineStr"/>
@@ -33311,7 +33311,7 @@
       <c r="F1012" t="inlineStr"/>
       <c r="G1012" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1012" t="inlineStr"/>
@@ -33379,7 +33379,7 @@
       <c r="F1014" t="inlineStr"/>
       <c r="G1014" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1014" t="inlineStr"/>
@@ -33413,7 +33413,7 @@
       <c r="F1015" t="inlineStr"/>
       <c r="G1015" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1015" t="inlineStr"/>
@@ -33447,7 +33447,7 @@
       <c r="F1016" t="inlineStr"/>
       <c r="G1016" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1016" t="inlineStr"/>
@@ -33511,7 +33511,7 @@
       <c r="F1018" t="inlineStr"/>
       <c r="G1018" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1018" t="inlineStr"/>
@@ -33545,7 +33545,7 @@
       <c r="F1019" t="inlineStr"/>
       <c r="G1019" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1019" t="inlineStr"/>
@@ -33579,7 +33579,7 @@
       <c r="F1020" t="inlineStr"/>
       <c r="G1020" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1020" t="inlineStr"/>
@@ -33613,7 +33613,7 @@
       <c r="F1021" t="inlineStr"/>
       <c r="G1021" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H1021" t="inlineStr"/>
@@ -33641,13 +33641,13 @@
       </c>
       <c r="E1022" t="inlineStr">
         <is>
-          <t>benutzer@domain.com, info@ringsidegym.ch, info@ringsidegym.ch</t>
+          <t>info@ringsidegym.ch</t>
         </is>
       </c>
       <c r="F1022" t="inlineStr"/>
       <c r="G1022" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@ringsidegym.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1022" t="inlineStr"/>
@@ -33741,7 +33741,7 @@
       <c r="F1025" t="inlineStr"/>
       <c r="G1025" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1025" t="inlineStr"/>
@@ -33805,7 +33805,7 @@
       <c r="F1027" t="inlineStr"/>
       <c r="G1027" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1027" t="inlineStr"/>
@@ -33839,7 +33839,7 @@
       <c r="F1028" t="inlineStr"/>
       <c r="G1028" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1028" t="inlineStr"/>
@@ -33873,7 +33873,7 @@
       <c r="F1029" t="inlineStr"/>
       <c r="G1029" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1029" t="inlineStr"/>
@@ -33907,7 +33907,7 @@
       <c r="F1030" t="inlineStr"/>
       <c r="G1030" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1030" t="inlineStr"/>
@@ -33941,7 +33941,7 @@
       <c r="F1031" t="inlineStr"/>
       <c r="G1031" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1031" t="inlineStr"/>
@@ -34039,7 +34039,7 @@
       <c r="F1034" t="inlineStr"/>
       <c r="G1034" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1034" t="inlineStr"/>
@@ -34073,7 +34073,7 @@
       <c r="F1035" t="inlineStr"/>
       <c r="G1035" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1035" t="inlineStr"/>
@@ -34137,7 +34137,7 @@
       <c r="F1037" t="inlineStr"/>
       <c r="G1037" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1037" t="inlineStr"/>
@@ -34171,7 +34171,7 @@
       <c r="F1038" t="inlineStr"/>
       <c r="G1038" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1038" t="inlineStr"/>
@@ -34205,7 +34205,7 @@
       <c r="F1039" t="inlineStr"/>
       <c r="G1039" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1039" t="inlineStr"/>
@@ -34233,13 +34233,13 @@
       </c>
       <c r="E1040" t="inlineStr">
         <is>
-          <t>support@webador.de, info@oneteamgym.ch</t>
+          <t>info@oneteamgym.ch</t>
         </is>
       </c>
       <c r="F1040" t="inlineStr"/>
       <c r="G1040" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@oneteamgym.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1040" t="inlineStr"/>
@@ -34297,13 +34297,13 @@
       </c>
       <c r="E1042" t="inlineStr">
         <is>
-          <t>info@klubdersportfreunde.ch, info@klubdersportfreunde.de</t>
+          <t>info@klubdersportfreunde.ch</t>
         </is>
       </c>
       <c r="F1042" t="inlineStr"/>
       <c r="G1042" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; info@klubdersportfreunde.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1042" t="inlineStr"/>
@@ -34337,7 +34337,7 @@
       <c r="F1043" t="inlineStr"/>
       <c r="G1043" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1043" t="inlineStr"/>
@@ -34371,7 +34371,7 @@
       <c r="F1044" t="inlineStr"/>
       <c r="G1044" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1044" t="inlineStr"/>
@@ -34405,7 +34405,7 @@
       <c r="F1045" t="inlineStr"/>
       <c r="G1045" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1045" t="inlineStr"/>
@@ -34529,7 +34529,7 @@
       <c r="F1049" t="inlineStr"/>
       <c r="G1049" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (malformed email cell: no usable address)</t>
         </is>
       </c>
       <c r="H1049" t="inlineStr"/>
@@ -34563,7 +34563,7 @@
       <c r="F1050" t="inlineStr"/>
       <c r="G1050" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EXCLUDED (day12 QA: placeholder/example domain)</t>
         </is>
       </c>
       <c r="H1050" t="inlineStr"/>
@@ -34597,7 +34597,7 @@
       <c r="F1051" t="inlineStr"/>
       <c r="G1051" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1051" t="inlineStr"/>
@@ -34661,7 +34661,7 @@
       <c r="F1053" t="inlineStr"/>
       <c r="G1053" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-26)</t>
         </is>
       </c>
       <c r="H1053" t="inlineStr"/>
@@ -34749,13 +34749,13 @@
       </c>
       <c r="E1056" t="inlineStr">
         <is>
-          <t>chaz.bjj.zh@gmail.com, info@mysite.com</t>
+          <t>chaz.bjj.zh@gmail.com</t>
         </is>
       </c>
       <c r="F1056" t="inlineStr"/>
       <c r="G1056" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | EMAIL FIXED (multi-address cell -&gt; chaz.bjj.zh@gmail.com; name-matched webmail)</t>
         </is>
       </c>
       <c r="H1056" t="inlineStr"/>
@@ -34789,6 +34789,544 @@
         </is>
       </c>
       <c r="H1057" t="inlineStr"/>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>L1947</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Portugal Judo Club</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>+351213884011</t>
+        </is>
+      </c>
+      <c r="E1058" t="inlineStr"/>
+      <c r="F1058" t="inlineStr"/>
+      <c r="G1058" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1058" t="inlineStr"/>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>L1952</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Crossfit Move On</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>+351934324900</t>
+        </is>
+      </c>
+      <c r="E1059" t="inlineStr"/>
+      <c r="F1059" t="inlineStr"/>
+      <c r="G1059" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1059" t="inlineStr"/>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>L1953</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>FACTORY GYM OF PHYSICAL</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>+351961781609</t>
+        </is>
+      </c>
+      <c r="E1060" t="inlineStr"/>
+      <c r="F1060" t="inlineStr"/>
+      <c r="G1060" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1060" t="inlineStr"/>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>L1955</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Zarka Jiu-Jitsu Academy</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>+351934937540</t>
+        </is>
+      </c>
+      <c r="E1061" t="inlineStr"/>
+      <c r="F1061" t="inlineStr"/>
+      <c r="G1061" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1061" t="inlineStr"/>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>L1956</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>BPT Arroios Nasser Camará</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>+351925393575</t>
+        </is>
+      </c>
+      <c r="E1062" t="inlineStr"/>
+      <c r="F1062" t="inlineStr"/>
+      <c r="G1062" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1062" t="inlineStr"/>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>L1957</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>RIO-SUL-BJJ</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>+351968269888</t>
+        </is>
+      </c>
+      <c r="E1063" t="inlineStr"/>
+      <c r="F1063" t="inlineStr">
+        <is>
+          <t>riosulventeira</t>
+        </is>
+      </c>
+      <c r="G1063" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | IG follow=ok dm=sent (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1063" t="inlineStr"/>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>L1958</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Connect Belt Team Brazilian Jiu Jitsu</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>+351926442202</t>
+        </is>
+      </c>
+      <c r="E1064" t="inlineStr"/>
+      <c r="F1064" t="inlineStr">
+        <is>
+          <t>connectbeltteamjiujitsu</t>
+        </is>
+      </c>
+      <c r="G1064" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | IG follow=ok dm=no-msg-btn (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1064" t="inlineStr"/>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>L1959</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>RIO21 - Academia de Jiu-jitsu</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>+351916995642</t>
+        </is>
+      </c>
+      <c r="E1065" t="inlineStr"/>
+      <c r="F1065" t="inlineStr">
+        <is>
+          <t>rio21.lisboa</t>
+        </is>
+      </c>
+      <c r="G1065" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | IG follow=no-btn dm=sent (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1065" t="inlineStr"/>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>L1960</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Fight Nation Santa Engracia</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>+351924093064</t>
+        </is>
+      </c>
+      <c r="E1066" t="inlineStr"/>
+      <c r="F1066" t="inlineStr"/>
+      <c r="G1066" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1066" t="inlineStr"/>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>L1963</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Hooked HPC</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>+41791251536</t>
+        </is>
+      </c>
+      <c r="E1067" t="inlineStr">
+        <is>
+          <t>hooked.hpc@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1067" t="inlineStr"/>
+      <c r="G1067" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1067" t="inlineStr"/>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>L1965</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>CrossFit Zurich</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>+41444310669</t>
+        </is>
+      </c>
+      <c r="E1068" t="inlineStr">
+        <is>
+          <t>info@crossfitzuerich.ch</t>
+        </is>
+      </c>
+      <c r="F1068" t="inlineStr"/>
+      <c r="G1068" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | EMAIL FIXED (multi-address cell -&gt; info@crossfitzuerich.ch; exact website domain) | COMPLETE: email sent (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1068" t="inlineStr"/>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>L1966</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Kensho Sports Baden</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>+41791757393</t>
+        </is>
+      </c>
+      <c r="E1069" t="inlineStr">
+        <is>
+          <t>info@kensho-sports.com</t>
+        </is>
+      </c>
+      <c r="F1069" t="inlineStr"/>
+      <c r="G1069" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | COMPLETE: email sent (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1069" t="inlineStr"/>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>L1968</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Ezinho BJJ | Jiu Jitsu Classes in Wallisellen</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>+41791975873</t>
+        </is>
+      </c>
+      <c r="E1070" t="inlineStr"/>
+      <c r="F1070" t="inlineStr">
+        <is>
+          <t>ezinho_bjj</t>
+        </is>
+      </c>
+      <c r="G1070" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26) | IG follow=ok dm=sent (Daily 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1070" t="inlineStr"/>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>L1969</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Judo und Ju-Jitsu Club Weisse Löwen Zürich</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>+41766994904</t>
+        </is>
+      </c>
+      <c r="E1071" t="inlineStr"/>
+      <c r="F1071" t="inlineStr"/>
+      <c r="G1071" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1071" t="inlineStr"/>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>L1970</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Van Led BJJ</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>+41764707818</t>
+        </is>
+      </c>
+      <c r="E1072" t="inlineStr"/>
+      <c r="F1072" t="inlineStr"/>
+      <c r="G1072" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1072" t="inlineStr"/>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>L1971</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Roger Gracie Brazilian Jiu Jitsu BJJ Zürich</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>+41763774216</t>
+        </is>
+      </c>
+      <c r="E1073" t="inlineStr"/>
+      <c r="F1073" t="inlineStr"/>
+      <c r="G1073" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1073" t="inlineStr"/>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>L1972</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>2Fight Zürich - Krav Maga Center</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>+41795401234</t>
+        </is>
+      </c>
+      <c r="E1074" t="inlineStr"/>
+      <c r="F1074" t="inlineStr"/>
+      <c r="G1074" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26)</t>
+        </is>
+      </c>
+      <c r="H1074" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
day12 final: WA pending list + tracker after ammo top-up (2026-10-26)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1074"/>
+  <dimension ref="A1:H1105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -35328,6 +35328,996 @@
       </c>
       <c r="H1074" t="inlineStr"/>
     </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>L1978</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Family Martial Arts Centre (Denton)</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>+447857989516</t>
+        </is>
+      </c>
+      <c r="E1075" t="inlineStr"/>
+      <c r="F1075" t="inlineStr"/>
+      <c r="G1075" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1075" t="inlineStr"/>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>L1980</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>GKKC Club</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>+447891653841</t>
+        </is>
+      </c>
+      <c r="E1076" t="inlineStr"/>
+      <c r="F1076" t="inlineStr"/>
+      <c r="G1076" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1076" t="inlineStr"/>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>L1983</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Ken Shu Dojo Karate Whitefield</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>+447886307454</t>
+        </is>
+      </c>
+      <c r="E1077" t="inlineStr"/>
+      <c r="F1077" t="inlineStr"/>
+      <c r="G1077" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1077" t="inlineStr"/>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>L1985</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Shins TKD Academy</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>+441618487426</t>
+        </is>
+      </c>
+      <c r="E1078" t="inlineStr">
+        <is>
+          <t>tw.shin@shinsacademytkd.co.uk</t>
+        </is>
+      </c>
+      <c r="F1078" t="inlineStr"/>
+      <c r="G1078" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1078" t="inlineStr"/>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>L1986</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Jeet Kune Do</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>+441619987062</t>
+        </is>
+      </c>
+      <c r="E1079" t="inlineStr"/>
+      <c r="F1079" t="inlineStr"/>
+      <c r="G1079" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1079" t="inlineStr"/>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>L1988</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Hybrid Mixed Martial Arts Academy</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>+447946813680</t>
+        </is>
+      </c>
+      <c r="E1080" t="inlineStr">
+        <is>
+          <t>jamie@hybridmma.academy</t>
+        </is>
+      </c>
+      <c r="F1080" t="inlineStr"/>
+      <c r="G1080" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1080" t="inlineStr"/>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>L1989</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Central Performance Centre - BJJ &amp; MMA in Stockport</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>+441617060660</t>
+        </is>
+      </c>
+      <c r="E1081" t="inlineStr">
+        <is>
+          <t>info@centralperformancecentre.co.uk</t>
+        </is>
+      </c>
+      <c r="F1081" t="inlineStr"/>
+      <c r="G1081" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1081" t="inlineStr"/>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>L1990</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Daywalkers MMA</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>+447946329261</t>
+        </is>
+      </c>
+      <c r="E1082" t="inlineStr"/>
+      <c r="F1082" t="inlineStr"/>
+      <c r="G1082" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1082" t="inlineStr"/>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>L1991</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>DEMAA</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>+447866952066</t>
+        </is>
+      </c>
+      <c r="E1083" t="inlineStr"/>
+      <c r="F1083" t="inlineStr"/>
+      <c r="G1083" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1083" t="inlineStr"/>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>L1992</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>AQF Sports | Boxing, MMA, Gym, Fitness Equipment &amp; Accessori</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>+441204704130</t>
+        </is>
+      </c>
+      <c r="E1084" t="inlineStr">
+        <is>
+          <t>info@aqfsports.co.uk</t>
+        </is>
+      </c>
+      <c r="F1084" t="inlineStr"/>
+      <c r="G1084" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1084" t="inlineStr"/>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>L1993</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>2 Technical Muay Thai</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>+447920002233</t>
+        </is>
+      </c>
+      <c r="E1085" t="inlineStr"/>
+      <c r="F1085" t="inlineStr"/>
+      <c r="G1085" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1085" t="inlineStr"/>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>L1994</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>SRMT</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>+447429496791</t>
+        </is>
+      </c>
+      <c r="E1086" t="inlineStr">
+        <is>
+          <t>info@rakhangmuaythai.co.uk</t>
+        </is>
+      </c>
+      <c r="F1086" t="inlineStr"/>
+      <c r="G1086" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1086" t="inlineStr"/>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>L1995</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>All Powers Gym</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>+447824996443</t>
+        </is>
+      </c>
+      <c r="E1087" t="inlineStr">
+        <is>
+          <t>allpowersgym@outlook.com</t>
+        </is>
+      </c>
+      <c r="F1087" t="inlineStr"/>
+      <c r="G1087" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1087" t="inlineStr"/>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>L1996</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Evade Martial Arts</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>+441457833987</t>
+        </is>
+      </c>
+      <c r="E1088" t="inlineStr">
+        <is>
+          <t>evademartialarts@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1088" t="inlineStr"/>
+      <c r="G1088" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1088" t="inlineStr"/>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>L1997</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Cherry Blossom BJJ &amp; Wellness</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>+447837006554</t>
+        </is>
+      </c>
+      <c r="E1089" t="inlineStr">
+        <is>
+          <t>cherryblossombjj@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1089" t="inlineStr"/>
+      <c r="G1089" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1089" t="inlineStr"/>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>L1998</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Manchester Brazilian Jiu-Jitsu: Bushido BJJ</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>+448606825876</t>
+        </is>
+      </c>
+      <c r="E1090" t="inlineStr">
+        <is>
+          <t>manchesterbjj@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1090" t="inlineStr"/>
+      <c r="G1090" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1090" t="inlineStr"/>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>L1999</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Grapple House BJJ</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>+447972194576</t>
+        </is>
+      </c>
+      <c r="E1091" t="inlineStr"/>
+      <c r="F1091" t="inlineStr"/>
+      <c r="G1091" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1091" t="inlineStr"/>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>L2000</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>UoM Jiu-Jitsu Club</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>+441615294444</t>
+        </is>
+      </c>
+      <c r="E1092" t="inlineStr"/>
+      <c r="F1092" t="inlineStr"/>
+      <c r="G1092" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1092" t="inlineStr"/>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>L2001</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Sale Ju-Jitsu Academy</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>+447469699121</t>
+        </is>
+      </c>
+      <c r="E1093" t="inlineStr">
+        <is>
+          <t>info@salejujitsu.co.uk</t>
+        </is>
+      </c>
+      <c r="F1093" t="inlineStr"/>
+      <c r="G1093" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1093" t="inlineStr"/>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>L2003</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Renzo Gracie NH</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>+446037772775</t>
+        </is>
+      </c>
+      <c r="E1094" t="inlineStr"/>
+      <c r="F1094" t="inlineStr"/>
+      <c r="G1094" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1094" t="inlineStr"/>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>L2004</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Manchester jujitsu club</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>UK</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>+447813897021</t>
+        </is>
+      </c>
+      <c r="E1095" t="inlineStr">
+        <is>
+          <t>johnshortt@manchesterjujitsuclub.com</t>
+        </is>
+      </c>
+      <c r="F1095" t="inlineStr"/>
+      <c r="G1095" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1095" t="inlineStr"/>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>L2007</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Dún Laoghaire Martial Arts</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>+353852214824</t>
+        </is>
+      </c>
+      <c r="E1096" t="inlineStr"/>
+      <c r="F1096" t="inlineStr"/>
+      <c r="G1096" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1096" t="inlineStr"/>
+    </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>L2009</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Brazier Jiu Jitsu</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>+353831304155</t>
+        </is>
+      </c>
+      <c r="E1097" t="inlineStr">
+        <is>
+          <t>hello.ie@brazierjiujitsu.com</t>
+        </is>
+      </c>
+      <c r="F1097" t="inlineStr"/>
+      <c r="G1097" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1097" t="inlineStr"/>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>L2010</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Tallaght Martial Arts And Fitness Centre</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>+353868388478</t>
+        </is>
+      </c>
+      <c r="E1098" t="inlineStr">
+        <is>
+          <t>tallaghtmartialarts@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1098" t="inlineStr"/>
+      <c r="G1098" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1098" t="inlineStr"/>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>L2011</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Silverback Jiu Jitsu Academy</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>+353872420647</t>
+        </is>
+      </c>
+      <c r="E1099" t="inlineStr">
+        <is>
+          <t>silverbackjiujitsuacademy@gmail.com</t>
+        </is>
+      </c>
+      <c r="F1099" t="inlineStr"/>
+      <c r="G1099" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1099" t="inlineStr"/>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>L2012</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Gracie Jiu-Jitsu Baldoyle | Ralph Gracie Ireland</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>+353851151123</t>
+        </is>
+      </c>
+      <c r="E1100" t="inlineStr"/>
+      <c r="F1100" t="inlineStr"/>
+      <c r="G1100" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1100" t="inlineStr"/>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>L2013</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Krav-Maga Bukan Dublin</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>+353838571853</t>
+        </is>
+      </c>
+      <c r="E1101" t="inlineStr">
+        <is>
+          <t>contact@kravmaga-ireland.com</t>
+        </is>
+      </c>
+      <c r="F1101" t="inlineStr"/>
+      <c r="G1101" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1101" t="inlineStr"/>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>L2014</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>UCD Karate</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1102" t="inlineStr">
+        <is>
+          <t>+35317163839</t>
+        </is>
+      </c>
+      <c r="E1102" t="inlineStr"/>
+      <c r="F1102" t="inlineStr"/>
+      <c r="G1102" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1102" t="inlineStr"/>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>L2018</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>St Matthews Boxing Club</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1103" t="inlineStr">
+        <is>
+          <t>+35316426008</t>
+        </is>
+      </c>
+      <c r="E1103" t="inlineStr"/>
+      <c r="F1103" t="inlineStr"/>
+      <c r="G1103" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1103" t="inlineStr"/>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>L2021</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Blackrock Health and Fitness</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1104" t="inlineStr">
+        <is>
+          <t>+353879141704</t>
+        </is>
+      </c>
+      <c r="E1104" t="inlineStr"/>
+      <c r="F1104" t="inlineStr"/>
+      <c r="G1104" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1104" t="inlineStr"/>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>L2022</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Cie Boxing Club</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Ireland</t>
+        </is>
+      </c>
+      <c r="D1105" t="inlineStr">
+        <is>
+          <t>+353852024171</t>
+        </is>
+      </c>
+      <c r="E1105" t="inlineStr"/>
+      <c r="F1105" t="inlineStr"/>
+      <c r="G1105" t="inlineStr">
+        <is>
+          <t>HUNTED (gmaps 2PM 2026-10-26-ammo-topup)</t>
+        </is>
+      </c>
+      <c r="H1105" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
day13 fix: re-mark 7 email-sent statuses clobbered by concurrent CSV writer (Gmail-verified)
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -31631,7 +31631,7 @@
       <c r="F942" t="inlineStr"/>
       <c r="G942" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H942" t="inlineStr"/>
@@ -31857,7 +31857,7 @@
       <c r="F949" t="inlineStr"/>
       <c r="G949" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H949" t="inlineStr"/>
@@ -37149,7 +37149,7 @@
       <c r="F1109" t="inlineStr"/>
       <c r="G1109" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H1109" t="inlineStr"/>
@@ -37745,7 +37745,7 @@
       </c>
       <c r="G1127" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27) | IG follow=ok dm=sent (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | IG follow=ok dm=sent (Daily 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H1127" t="inlineStr"/>
@@ -38043,7 +38043,7 @@
       <c r="F1136" t="inlineStr"/>
       <c r="G1136" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H1136" t="inlineStr"/>
@@ -38187,7 +38187,7 @@
       </c>
       <c r="G1140" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27) | IG profile not found (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | IG profile not found (Daily 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H1140" t="inlineStr"/>
@@ -38285,7 +38285,7 @@
       <c r="F1143" t="inlineStr"/>
       <c r="G1143" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H1143" t="inlineStr"/>

</xml_diff>

<commit_message>
day13 final: 100 emails (97+3 topup), 3 bounces marked failed, 71 IG
</commit_message>
<xml_diff>
--- a/WA_Pending_List.xlsx
+++ b/WA_Pending_List.xlsx
@@ -11563,7 +11563,7 @@
       <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EMAIL VERIFIED (webmail, name-matched)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | EMAIL VERIFIED (webmail, name-matched) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H332" t="inlineStr"/>
@@ -12363,7 +12363,7 @@
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-23) | EMAIL VERIFIED (webmail, name-matched) | IG follow=clicked dm=sent (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-23) | EMAIL VERIFIED (webmail, name-matched) | IG follow=clicked dm=sent (Daily 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
         </is>
       </c>
       <c r="H356" t="inlineStr"/>
@@ -33851,7 +33851,7 @@
       </c>
       <c r="G1010" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) | COMPLETE: email sent (Daily 2026-10-27) | IG profile not found (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-25-ammo-topup) |  | IG profile not found (Daily 2026-10-27) | EMAIL FAILED (Daily 2026-10-27): domain not found (Vera bjj kids)</t>
         </is>
       </c>
       <c r="H1010" t="inlineStr"/>
@@ -37907,7 +37907,7 @@
       <c r="F1132" t="inlineStr"/>
       <c r="G1132" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) | EMAIL FAILED (Daily 2026-10-27): recipient-not-registered (Blue Siytangco Taiji Kungfu)</t>
         </is>
       </c>
       <c r="H1132" t="inlineStr"/>
@@ -39351,7 +39351,7 @@
       </c>
       <c r="G1174" t="inlineStr">
         <is>
-          <t>HUNTED (gmaps 2PM 2026-10-27) | COMPLETE: email sent (Daily 2026-10-27) | IG follow=ok dm=sent (Daily 2026-10-27)</t>
+          <t>HUNTED (gmaps 2PM 2026-10-27) |  | IG follow=ok dm=sent (Daily 2026-10-27) | EMAIL FAILED (Daily 2026-10-27): address not found (Windy City Boxing)</t>
         </is>
       </c>
       <c r="H1174" t="inlineStr"/>

</xml_diff>